<commit_message>
Update Naver Webtoon Series mapping
</commit_message>
<xml_diff>
--- a/data/adult_login_required_webtoons_v2.xlsx
+++ b/data/adult_login_required_webtoons_v2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK53"/>
+  <dimension ref="A1:AK54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -634,7 +634,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-22 11:40:58</t>
+          <t>2026-06-29 13:06:01</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-22 11:40:59</t>
+          <t>2026-06-29 13:06:01</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -910,7 +910,7 @@
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-22 11:40:59</t>
+          <t>2026-06-29 13:06:02</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:00</t>
+          <t>2026-06-29 13:06:02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:00</t>
+          <t>2026-06-29 13:06:03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:01</t>
+          <t>2026-06-29 13:06:03</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:02</t>
+          <t>2026-06-29 13:06:05</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:02</t>
+          <t>2026-06-29 13:06:05</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:02</t>
+          <t>2026-06-29 13:06:05</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:03</t>
+          <t>2026-06-29 13:06:05</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:03</t>
+          <t>2026-06-29 13:06:06</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -2341,26 +2341,26 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>축살</t>
+          <t>화분</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=840184&amp;tab=tue</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=851671&amp;tab=tue</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>840184</t>
+          <t>851671</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:03</t>
+          <t>2026-06-29 13:06:06</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2388,21 +2388,21 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>축살</t>
+          <t>화분</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>축살 (총 51화/미완결)</t>
+          <t>화분 (총 5화/미완결)</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>총 51화/미완결</t>
+          <t>총 5화/미완결</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -2411,30 +2411,30 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>평점 9.9 | 장성준 장성준 | 2026.05.11. | 총51화/미완결 | 전화 무료</t>
+          <t>평점 10.0 | 쿼시 쿼시 | 2026.06.15. | 총5화/미완결 | 1화 무료</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>평점 9.9 | 장성준 장성준 | 2026.05.11. | 총51화/미완결 | 전화 무료</t>
+          <t>평점 10.0 | 쿼시 쿼시 | 2026.06.15. | 총5화/미완결 | 1화 무료</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=12763164</t>
+          <t>https://series.naver.com/comic/detail.series?productNo=14284647</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>12763164</t>
+          <t>14284647</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>축살 (총 51화/미완결)
+          <t>화분 (총 5화/미완결)
 평점
-9.9 | 장성준 장성준 | 2026.05.11. | 총51화/미완결 | 전화 무료
-귀신이 나온다는 이유로 아무도 찾지 않는 버려진 마을이 된 타악리...그곳을 미스테리X파일 제작팀이 관심을 갖고 찾아간다. 그러나 기다리는 것은 당시 사건으로 죽은 귀신과, 염매라는 사악한 주술을 통해 살아 있는 악귀가 ..</t>
+10.0 | 쿼시 쿼시 | 2026.06.15. | 총5화/미완결 | 1화 무료
+버림받는 것이 무서운 여자와 그런 그녀가 무섭게 느껴지는 남자. 오래된 인연으로 시작된 사랑은 다정함의 얼굴을 한 집착이 되어, 두 사람의 일상과 마음을 서서히 갉아먹어 간다.우리 사랑은, 어디서부터 잘못된거지..?</t>
         </is>
       </c>
       <c r="Y13" t="b">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:04</t>
+          <t>2026-06-29 13:06:06</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -2653,26 +2653,26 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>화분</t>
+          <t>포 더 퀸덤</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=851671&amp;tab=tue</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=812414&amp;tab=tue</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>851671</t>
+          <t>812414</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:04</t>
+          <t>2026-06-29 13:06:07</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2700,21 +2700,21 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>화분</t>
+          <t>포 더 퀸덤</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>화분 (총 5화/미완결)</t>
+          <t>포 더 퀸덤 (총 128화/미완결)</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>총 5화/미완결</t>
+          <t>총 128화/미완결</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>5</v>
+        <v>128</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -2723,181 +2723,25 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>평점 10.0 | 쿼시 쿼시 | 2026.06.15. | 총5화/미완결 | 1화 무료</t>
+          <t>평점 9.0 | 로즈옹 로즈옹 | 2026.06.15. | 총128화/미완결 | 123화 무료</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>평점 10.0 | 쿼시 쿼시 | 2026.06.15. | 총5화/미완결 | 1화 무료</t>
+          <t>평점 9.0 | 로즈옹 로즈옹 | 2026.06.15. | 총128화/미완결 | 123화 무료</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=14284647</t>
+          <t>https://series.naver.com/comic/detail.series?productNo=9895056</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>14284647</t>
+          <t>9895056</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
-        <is>
-          <t>화분 (총 5화/미완결)
-평점
-10.0 | 쿼시 쿼시 | 2026.06.15. | 총5화/미완결 | 1화 무료
-버림받는 것이 무서운 여자와 그런 그녀가 무섭게 느껴지는 남자. 오래된 인연으로 시작된 사랑은 다정함의 얼굴을 한 집착이 되어, 두 사람의 일상과 마음을 서서히 갉아먹어 간다.우리 사랑은, 어디서부터 잘못된거지..?</t>
-        </is>
-      </c>
-      <c r="Y15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI15" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ15" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>tue</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>화</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>79</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>포 더 퀸덤</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=812414&amp;tab=tue</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>812414</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:05</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="b">
-        <v>1</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>tue</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>tue</t>
-        </is>
-      </c>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>포 더 퀸덤</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>포 더 퀸덤 (총 128화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>총 128화/미완결</t>
-        </is>
-      </c>
-      <c r="R16" t="n">
-        <v>128</v>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>평점 9.0 | 로즈옹 로즈옹 | 2026.06.15. | 총128화/미완결 | 123화 무료</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>평점 9.0 | 로즈옹 로즈옹 | 2026.06.15. | 총128화/미완결 | 123화 무료</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=9895056</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>9895056</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
         <is>
           <t>포 더 퀸덤 (총 128화/미완결)
 평점
@@ -2905,6 +2749,162 @@
 악마 아벨은 인간 여자 연리에게 사랑하는 형, 카인을 잃고 만다.분노에 가득 차 연리를 찾아간 아벨은 사랑에 빠지는 금총알을 맞게 되면서, 연리에게 끓어오르는 사랑을 느끼게 되는데…그는 과연 형제의 복수를 택할 것인가..</t>
         </is>
       </c>
+      <c r="Y15" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tue</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>화</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>100</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>연애 못하면 사망</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=834175&amp;tab=tue</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>834175</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:07</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>tue</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>tue</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>연애 못하면 사망</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>연애 못하면 사망 (총 85화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>총 85화/미완결</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>85</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 홍치 홍치 | 2026.06.15. | 총85화/미완결 | 80화 무료</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 홍치 홍치 | 2026.06.15. | 총85화/미완결 | 80화 무료</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=11845281</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>11845281</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>연애 못하면 사망 (총 85화/미완결)
+평점
+10.0 | 홍치 홍치 | 2026.06.15. | 총85화/미완결 | 80화 무료
+111세 덕순 F&amp;B의 회장 김덕순은 죽기 직전 마지막 소원으로 첫사랑 왕종열과의 불꽃 같은 사랑을 하게 해달라 빌고 25세 김도희라는 여자의 몸에서 깨어난다. 그러나 마지막 소원을 이루기 위해 종열을 향해 달려가던 덕순..</t>
+        </is>
+      </c>
       <c r="Y16" t="b">
         <v>0</v>
       </c>
@@ -2912,31 +2912,37 @@
         <v>1</v>
       </c>
       <c r="AA16" t="n">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+          <t>title_contains,author_exact_or_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>review_needed</t>
+          <t>matched</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>non_compilation_but_download_not_ok</t>
+          <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
       <c r="AE16" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>37만</t>
+        </is>
+      </c>
+      <c r="AG16" t="n">
+        <v>370000</v>
+      </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
@@ -2949,7 +2955,7 @@
       </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2971,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2984,7 +2990,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:06</t>
+          <t>2026-06-29 13:06:08</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -3105,7 +3111,7 @@
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3146,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:06</t>
+          <t>2026-06-29 13:06:08</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -3261,7 +3267,7 @@
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3283,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -3296,7 +3302,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:06</t>
+          <t>2026-06-29 13:06:08</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -3423,7 +3429,7 @@
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3445,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -3458,7 +3464,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:07</t>
+          <t>2026-06-29 13:06:09</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -3579,7 +3585,7 @@
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3620,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:07</t>
+          <t>2026-06-29 13:06:09</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3741,7 +3747,7 @@
       </c>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3763,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -3776,7 +3782,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:07</t>
+          <t>2026-06-29 13:06:09</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3897,7 +3903,7 @@
       </c>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3919,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -3932,7 +3938,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:08</t>
+          <t>2026-06-29 13:06:10</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -4053,7 +4059,7 @@
       </c>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4094,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:10</t>
+          <t>2026-06-29 13:06:11</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -4209,7 +4215,7 @@
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -4225,26 +4231,26 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>당신의 살인을 위하여</t>
+          <t>당신에게 얽힌 채</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=836066&amp;tab=thu</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=849879&amp;tab=thu</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>836066</t>
+          <t>849879</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:11</t>
+          <t>2026-06-29 13:06:12</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -4272,21 +4278,21 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>당신의 살인을 위하여</t>
+          <t>당신에게 얽힌 채</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>당신의 살인을 위하여 (총 70화/미완결)</t>
+          <t>당신에게 얽힌 채 (총 10화/미완결)</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>총 70화/미완결</t>
+          <t>총 10화/미완결</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -4295,181 +4301,25 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>평점 9.9 | 세윤 징크 | 2026.06.17. | 총70화/미완결 | 전화 무료</t>
+          <t>평점 10.0 | Nicole Knight, 유다 danah789 | 2026.06.17. | 총10화/미완결 | 5화 무료</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>평점 9.9 | 세윤 징크 | 2026.06.17. | 총70화/미완결 | 전화 무료</t>
+          <t>평점 10.0 | Nicole Knight, 유다 danah789 | 2026.06.17. | 총10화/미완결 | 5화 무료</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=12161861</t>
+          <t>https://series.naver.com/comic/detail.series?productNo=14041685</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>12161861</t>
+          <t>14041685</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
-        <is>
-          <t>당신의 살인을 위하여 (총 70화/미완결)
-평점
-9.9 | 세윤 징크 | 2026.06.17. | 총70화/미완결 | 전화 무료
-자신을 억누르고 사는 초등학교 교사 고기정은 학부모에게 시달리다 근처 변호사를 찾아간다.그러나 찾아간 변호사 오인섭은 연쇄살인마였는데..</t>
-        </is>
-      </c>
-      <c r="Y25" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB25" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC25" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD25" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI25" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ25" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK25" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>thu</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>목</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>34</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>당신에게 얽힌 채</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=849879&amp;tab=thu</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>849879</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:11</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="b">
-        <v>1</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>thu</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>thu</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>당신에게 얽힌 채</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>당신에게 얽힌 채 (총 10화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>총 10화/미완결</t>
-        </is>
-      </c>
-      <c r="R26" t="n">
-        <v>10</v>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>평점 10.0 | Nicole Knight, 유다 danah789 | 2026.06.17. | 총10화/미완결 | 5화 무료</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>평점 10.0 | Nicole Knight, 유다 danah789 | 2026.06.17. | 총10화/미완결 | 5화 무료</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=14041685</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>14041685</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
         <is>
           <t>당신에게 얽힌 채 (총 10화/미완결)
 평점
@@ -4477,155 +4327,155 @@
 상속자가 아닌 복종하는 존재로 길러진 에이바 모레티. 뉴욕에서 가장 강력한 마피아 가문의 막내딸인 그녀는 ‘집안의 사고뭉치’라는 오명을 벗고 자신의 자리를 찾기 위해 분투한다.그러던 어느 날 밤, 낯선 남자와 보낸 뜨..</t>
         </is>
       </c>
-      <c r="Y26" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z26" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA26" t="n">
+      <c r="Y25" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA25" t="n">
         <v>105</v>
       </c>
-      <c r="AB26" t="inlineStr">
+      <c r="AB25" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC26" t="inlineStr">
+      <c r="AC25" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD26" t="inlineStr">
+      <c r="AD25" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr">
+      <c r="AE25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI26" t="inlineStr">
+      <c r="AI25" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ26" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK26" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ25" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>thu</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>목</t>
         </is>
       </c>
-      <c r="C27" t="n">
-        <v>76</v>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="C26" t="n">
+        <v>74</v>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>휴먼 웨어러블</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=845460&amp;tab=thu</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>845460</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:13</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="b">
-        <v>1</v>
-      </c>
-      <c r="J27" t="inlineStr">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:14</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
         <is>
           <t>thu</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>thu</t>
         </is>
       </c>
-      <c r="N27" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="inlineStr">
         <is>
           <t>휴먼 웨어러블</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>휴먼 웨어러블 (총 30화/미완결)</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>총 30화/미완결</t>
         </is>
       </c>
-      <c r="R27" t="n">
+      <c r="R26" t="n">
         <v>30</v>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>평점 9.9 | 쥬타인 쥬타인 | 2026.06.03. | 총30화/미완결 | 27화 무료</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>평점 9.9 | 쥬타인 쥬타인 | 2026.06.03. | 총30화/미완결 | 27화 무료</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=13481722</t>
         </is>
       </c>
-      <c r="W27" t="inlineStr">
+      <c r="W26" t="inlineStr">
         <is>
           <t>13481722</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>휴먼 웨어러블 (총 30화/미완결)
 평점
@@ -4633,6 +4483,162 @@
 꿈의 무대, 패션 서바이벌 &lt;휴먼 웨어러블&gt;.고아 출신이지만 명문 ‘순백패션예술학교’를 거쳐 올라온 학생들.이 무대에서 인생 역전의 주인공이 탄생한다—…그런데 무언가, 이상하게 흘러가기 시작했다.</t>
         </is>
       </c>
+      <c r="Y26" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ26" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>thu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>목</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>102</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>운명해주세요</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=835004&amp;tab=thu</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>835004</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:14</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>thu</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>thu</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>운명해주세요</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>운명해주세요 (총 53화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>총 53화/미완결</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>53</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 노뱀 노뱀 | 2025.12.24. | 총53화/미완결 | 전화 무료</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 노뱀 노뱀 | 2025.12.24. | 총53화/미완결 | 전화 무료</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=11990945</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>11990945</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>운명해주세요 (총 53화/미완결)
+평점
+10.0 | 노뱀 노뱀 | 2025.12.24. | 총53화/미완결 | 전화 무료
+무수한 고난을 알코올의 힘으로 씩씩하게 이겨내는 청년 백수 해솔.그런 해솔의 앞에 13년 만에 나타난 수상한 속내의 하현.둘 중 하나가 죽어야만 살 수 있는 해솔과 하현의 저세상 로맨스!</t>
+        </is>
+      </c>
       <c r="Y27" t="b">
         <v>0</v>
       </c>
@@ -4649,27 +4655,33 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>review_needed</t>
+          <t>matched</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>non_compilation_but_download_not_ok</t>
+          <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
       <c r="AE27" t="n">
         <v>1</v>
       </c>
-      <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>12.7만</t>
+        </is>
+      </c>
+      <c r="AG27" t="n">
+        <v>127000</v>
+      </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AI27" t="inlineStr">
         <is>
-          <t>reused_existing_product_no</t>
+          <t>searched_series</t>
         </is>
       </c>
       <c r="AJ27" t="b">
@@ -4677,7 +4689,7 @@
       </c>
       <c r="AK27" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4705,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -4712,7 +4724,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:14</t>
+          <t>2026-06-29 13:06:15</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -4833,7 +4845,7 @@
       </c>
       <c r="AK28" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4880,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:15</t>
+          <t>2026-06-29 13:06:15</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -4995,7 +5007,7 @@
       </c>
       <c r="AK29" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5042,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:15</t>
+          <t>2026-06-29 13:06:15</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -5151,7 +5163,7 @@
       </c>
       <c r="AK30" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5198,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:15</t>
+          <t>2026-06-29 13:06:15</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -5307,7 +5319,7 @@
       </c>
       <c r="AK31" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5342,7 +5354,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:16</t>
+          <t>2026-06-29 13:06:16</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -5463,7 +5475,7 @@
       </c>
       <c r="AK32" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5510,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:16</t>
+          <t>2026-06-29 13:06:16</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -5625,7 +5637,7 @@
       </c>
       <c r="AK33" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5672,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:17</t>
+          <t>2026-06-29 13:06:17</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -5787,7 +5799,7 @@
       </c>
       <c r="AK34" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5815,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -5822,7 +5834,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:18</t>
+          <t>2026-06-29 13:06:17</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -5943,7 +5955,7 @@
       </c>
       <c r="AK35" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5971,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -5978,7 +5990,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:18</t>
+          <t>2026-06-29 13:06:17</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -6099,7 +6111,7 @@
       </c>
       <c r="AK36" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -6115,26 +6127,26 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>완벽한 게 다인</t>
+          <t>나의 모르는 여자친구</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=841767&amp;tab=fri</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=841923&amp;tab=fri</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>841767</t>
+          <t>841923</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:20</t>
+          <t>2026-06-29 13:06:19</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -6162,21 +6174,21 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>완벽한 게 다인</t>
+          <t>나의 모르는 여자친구</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>완벽한 게 다인 (총 46화/미완결)</t>
+          <t>나의 모르는 여자친구 (총 41화/미완결)</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>총 46화/미완결</t>
+          <t>총 41화/미완결</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -6185,26 +6197,26 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>평점 10.0 | 은솔 재림 | 2026.06.04. | 총46화/미완결 | 41화 무료</t>
+          <t>평점 9.9 | 이정빈 이정빈 | 2026.06.04. | 총41화/미완결 | 36화 무료</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=13009203</t>
+          <t>https://series.naver.com/comic/detail.series?productNo=13025901</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>13009203</t>
+          <t>13025901</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>완벽한 게 다인 (총 46화/미완결)
+          <t>나의 모르는 여자친구 (총 41화/미완결)
 평점
-10.0 | 은솔 재림 | 2026.06.04. | 총46화/미완결 | 41화 무료
-매사에 열심히, 열정적인 학창시절을 살아온 대학 새내기 김다인은 성적, 교우관계, 스펙 모든 것이 완벽한 캠퍼스 라이프를 꿈꾼다.하지만 다인은 자신과 이름이 같지만 자신과 다르게 '완벽한 외모와 인성을 겸비한' 강다인..</t>
+9.9 | 이정빈 이정빈 | 2026.06.04. | 총41화/미완결 | 36화 무료
+눈 떠보니 아이돌의 여자친구가 되어있다?! 평범한 삶을 추구하는 대학생 ‘해나’는 인기 아이돌 ‘은하‘와의 거짓 열애설로 일상에 금이 갈 위기를 맞는다.</t>
         </is>
       </c>
       <c r="Y37" t="b">
@@ -6236,11 +6248,11 @@
       </c>
       <c r="AF37" t="inlineStr">
         <is>
-          <t>25.8만</t>
+          <t>7.8만</t>
         </is>
       </c>
       <c r="AG37" t="n">
-        <v>258000</v>
+        <v>78000</v>
       </c>
       <c r="AH37" t="inlineStr">
         <is>
@@ -6257,7 +6269,7 @@
       </c>
       <c r="AK37" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6304,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:21</t>
+          <t>2026-06-29 13:06:19</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -6412,7 +6424,7 @@
       </c>
       <c r="AK38" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6459,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:21</t>
+          <t>2026-06-29 13:06:19</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -6568,7 +6580,7 @@
       </c>
       <c r="AK39" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6596,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -6603,7 +6615,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:21</t>
+          <t>2026-06-29 13:06:19</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -6724,7 +6736,7 @@
       </c>
       <c r="AK40" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -6759,7 +6771,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:21</t>
+          <t>2026-06-29 13:06:19</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -6880,7 +6892,7 @@
       </c>
       <c r="AK41" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -6896,7 +6908,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -6915,7 +6927,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:23</t>
+          <t>2026-06-29 13:06:20</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -7036,7 +7048,7 @@
       </c>
       <c r="AK42" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7064,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -7071,7 +7083,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:23</t>
+          <t>2026-06-29 13:06:20</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -7192,7 +7204,7 @@
       </c>
       <c r="AK43" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
@@ -7208,7 +7220,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -7227,7 +7239,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:23</t>
+          <t>2026-06-29 13:06:20</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -7348,42 +7360,42 @@
       </c>
       <c r="AK44" t="inlineStr">
         <is>
-          <t>2026-06-22 12:22:39</t>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sun</t>
+          <t>sat</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2회차 환관이 남성을 되찾음</t>
+          <t>데스루프</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=832566&amp;tab=sun</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=852086&amp;tab=sat</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>832566</t>
+          <t>852086</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-06-22 11:41:26</t>
+          <t>2026-06-29 13:06:21</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -7398,61 +7410,217 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
+          <t>sat</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>sat</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>1</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>데스루프</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>데스루프 (총 6화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>총 6화/미완결</t>
+        </is>
+      </c>
+      <c r="R45" t="n">
+        <v>6</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>평점 8.3 | 은삼 은삼 | 2026.06.26. | 총6화/미완결 | 1화 무료</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>평점 8.3 | 은삼 은삼 | 2026.06.26. | 총6화/미완결 | 1화 무료</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=14366954</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>14366954</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>데스루프 (총 6화/미완결)
+평점
+8.3 | 은삼 은삼 | 2026.06.26. | 총6화/미완결 | 1화 무료
+정신을 차려 보니 지하 창고에 갇힌 주인공 홍연화.연화는 자신을 가둔 남성에게 여러 번 끔찍한 죽음을 맞이하지만, 계속해서 시간이 반복된다.겨우 그곳을 빠져나오지만 그녀 앞에 마주한 것은 끔찍하게 생긴 괴물.과연 그녀..</t>
+        </is>
+      </c>
+      <c r="Y45" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF45" t="inlineStr"/>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>searched_series</t>
+        </is>
+      </c>
+      <c r="AJ45" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2회차 환관이 남성을 되찾음</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=832566&amp;tab=sun</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>832566</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:23</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="b">
+        <v>1</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N45" t="n">
-        <v>1</v>
-      </c>
-      <c r="O45" t="inlineStr">
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>1</v>
+      </c>
+      <c r="O46" t="inlineStr">
         <is>
           <t>2회차 환관이 남성을 되찾음</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="P46" t="inlineStr">
         <is>
           <t>2회차 환관이 남성을 되찾음 (총 93화/미완결)</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="Q46" t="inlineStr">
         <is>
           <t>총 93화/미완결</t>
         </is>
       </c>
-      <c r="R45" t="n">
+      <c r="R46" t="n">
         <v>93</v>
       </c>
-      <c r="S45" t="inlineStr">
+      <c r="S46" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T45" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>평점 9.6 | LICO, 노빠꾸맨 포스 스튜디오 | 2026.06.13. | 총93화/미완결 | 89화 무료</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>평점 9.6 | LICO, 노빠꾸맨 포스 스튜디오 | 2026.06.13. | 총93화/미완결 | 89화 무료</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
+      <c r="V46" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=11636787</t>
         </is>
       </c>
-      <c r="W45" t="inlineStr">
+      <c r="W46" t="inlineStr">
         <is>
           <t>11636787</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>2회차 환관이 남성을 되찾음 (총 93화/미완결)
 평점
@@ -7460,310 +7628,310 @@
 제국의 국정을 마음대로 주무르는 비선실세 환관, 이철수.절대 권력에 돈 많고, 무공까지 강하지만.. 그게 무슨 의미가 있지? '그걸' 못하는데!!환생대법을 통해, 고자가 되기 전으로 회귀한 철수의 목표는 하나다.알파메일이 되..</t>
         </is>
       </c>
-      <c r="Y45" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z45" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA45" t="n">
+      <c r="Y46" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z46" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA46" t="n">
         <v>105</v>
       </c>
-      <c r="AB45" t="inlineStr">
+      <c r="AB46" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC45" t="inlineStr">
+      <c r="AC46" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD45" t="inlineStr">
+      <c r="AD46" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE45" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF45" t="inlineStr"/>
-      <c r="AG45" t="inlineStr"/>
-      <c r="AH45" t="inlineStr">
+      <c r="AE46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF46" t="inlineStr"/>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI45" t="inlineStr">
+      <c r="AI46" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ45" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK45" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ46" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C46" t="n">
-        <v>5</v>
-      </c>
-      <c r="D46" t="inlineStr">
+      <c r="C47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>시루/24/1km</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=850068&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>850068</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:26</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="b">
-        <v>1</v>
-      </c>
-      <c r="J46" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:23</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="b">
+        <v>1</v>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N46" t="n">
-        <v>1</v>
-      </c>
-      <c r="O46" t="inlineStr">
+      <c r="N47" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" t="inlineStr">
         <is>
           <t>19금 시루/24/1km</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>19금 시루/24/1km (총 12화/미완결)</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
+      <c r="Q47" t="inlineStr">
         <is>
           <t>총 12화/미완결</t>
         </is>
       </c>
-      <c r="R46" t="n">
+      <c r="R47" t="n">
         <v>12</v>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S47" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T47" t="inlineStr">
         <is>
           <t>평점 10.0 | 6M 941 | 2026.06.13. | 총12화/미완결 | 7화 무료</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U47" t="inlineStr">
         <is>
           <t>평점 10.0 | 6M 941 | 2026.06.13. | 총12화/미완결 | 7화 무료</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="V47" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14081030</t>
         </is>
       </c>
-      <c r="W46" t="inlineStr">
+      <c r="W47" t="inlineStr">
         <is>
           <t>14081030</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>19금 시루/24/1km (총 12화/미완결)
 평점
 10.0 | 6M 941 | 2026.06.13. | 총12화/미완결 | 7화 무료</t>
         </is>
       </c>
-      <c r="Y46" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z46" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA46" t="n">
+      <c r="Y47" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z47" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA47" t="n">
         <v>105</v>
       </c>
-      <c r="AB46" t="inlineStr">
+      <c r="AB47" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC46" t="inlineStr">
+      <c r="AC47" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD46" t="inlineStr">
+      <c r="AD47" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE46" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF46" t="inlineStr"/>
-      <c r="AG46" t="inlineStr"/>
-      <c r="AH46" t="inlineStr">
+      <c r="AE47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF47" t="inlineStr"/>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI46" t="inlineStr">
+      <c r="AI47" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ46" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK46" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ47" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C47" t="n">
-        <v>10</v>
-      </c>
-      <c r="D47" t="inlineStr">
+      <c r="C48" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>어린 아내와 나쁜 짓</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=851385&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>851385</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:26</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="b">
-        <v>1</v>
-      </c>
-      <c r="J47" t="inlineStr">
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:23</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="b">
+        <v>1</v>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N47" t="n">
-        <v>1</v>
-      </c>
-      <c r="O47" t="inlineStr">
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t>어린 아내와 나쁜 짓</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>어린 아내와 나쁜 짓 (총 8화/미완결)</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
+      <c r="Q48" t="inlineStr">
         <is>
           <t>총 8화/미완결</t>
         </is>
       </c>
-      <c r="R47" t="n">
+      <c r="R48" t="n">
         <v>8</v>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="S48" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>평점 9.9 | 이리와, 무멘 83 | 2026.06.13. | 총8화/미완결 | 2화 무료</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>평점 9.9 | 이리와, 무멘 83 | 2026.06.13. | 총8화/미완결 | 2화 무료</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr">
+      <c r="V48" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14245757</t>
         </is>
       </c>
-      <c r="W47" t="inlineStr">
+      <c r="W48" t="inlineStr">
         <is>
           <t>14245757</t>
         </is>
       </c>
-      <c r="X47" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>어린 아내와 나쁜 짓 (총 8화/미완결)
 평점
@@ -7771,155 +7939,155 @@
 절망의 끝에서 나를 구원해준 남자, 범도건.작고 지켜야할 애기님이라며 내 고백을 짓밞았던 그때와는 다르게...이 남자, 남편 역할을 해도 너무 잘한다.낮에는 세상 든든한 보호자이던 그가 밤만 되면 맹수처럼 집착하며 나를 ..</t>
         </is>
       </c>
-      <c r="Y47" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z47" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA47" t="n">
+      <c r="Y48" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z48" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA48" t="n">
         <v>105</v>
       </c>
-      <c r="AB47" t="inlineStr">
+      <c r="AB48" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC47" t="inlineStr">
+      <c r="AC48" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD47" t="inlineStr">
+      <c r="AD48" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE47" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF47" t="inlineStr"/>
-      <c r="AG47" t="inlineStr"/>
-      <c r="AH47" t="inlineStr">
+      <c r="AE48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF48" t="inlineStr"/>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI47" t="inlineStr">
+      <c r="AI48" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ47" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK47" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ48" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C48" t="n">
+      <c r="C49" t="n">
         <v>12</v>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>유쾌한 신</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=846053&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>846053</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:26</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="b">
-        <v>1</v>
-      </c>
-      <c r="J48" t="inlineStr">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:23</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="b">
+        <v>1</v>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
         <is>
           <t>wed,sun</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>wed,sun</t>
         </is>
       </c>
-      <c r="N48" t="n">
+      <c r="N49" t="n">
         <v>2</v>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="O49" t="inlineStr">
         <is>
           <t>당신의 유쾌한 주말</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="P49" t="inlineStr">
         <is>
           <t>당신의 유쾌한 주말 (총 19화/미완결)</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr">
+      <c r="Q49" t="inlineStr">
         <is>
           <t>총 19화/미완결</t>
         </is>
       </c>
-      <c r="R48" t="n">
+      <c r="R49" t="n">
         <v>19</v>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S49" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="T49" t="inlineStr">
         <is>
           <t>평점 9.4 | 김수영 김수영 | 2010.04.20. | 총19화/미완결</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>평점 9.4 | 김수영 김수영 | 2010.04.20. | 총19화/미완결</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
+      <c r="V49" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=57402</t>
         </is>
       </c>
-      <c r="W48" t="inlineStr">
+      <c r="W49" t="inlineStr">
         <is>
           <t>57402</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>당신의 유쾌한 주말 (총 19화/미완결)
 평점
@@ -7927,161 +8095,161 @@
 화창한 토욜 인형을 잔뜩 가지고 나온 남자는 오는 손님 쫓고 가는 손님은 거들 떠 보지도 않는다. 사실 이 남자는 인형 만들기에 빠져 연재가 짤린 만화가였으니...</t>
         </is>
       </c>
-      <c r="Y48" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z48" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA48" t="n">
+      <c r="Y49" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z49" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA49" t="n">
         <v>30</v>
       </c>
-      <c r="AB48" t="inlineStr">
+      <c r="AB49" t="inlineStr">
         <is>
           <t>bonus_total_episode_info,bonus_rank_2</t>
         </is>
       </c>
-      <c r="AC48" t="inlineStr">
+      <c r="AC49" t="inlineStr">
         <is>
           <t>matched</t>
         </is>
       </c>
-      <c r="AD48" t="inlineStr">
+      <c r="AD49" t="inlineStr">
         <is>
           <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
-      <c r="AE48" t="n">
+      <c r="AE49" t="n">
         <v>2</v>
       </c>
-      <c r="AF48" t="inlineStr">
+      <c r="AF49" t="inlineStr">
         <is>
           <t>3.8천</t>
         </is>
       </c>
-      <c r="AG48" t="n">
+      <c r="AG49" t="n">
         <v>3800</v>
       </c>
-      <c r="AH48" t="inlineStr">
+      <c r="AH49" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="AI48" t="inlineStr">
+      <c r="AI49" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ48" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK48" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ49" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C49" t="n">
+      <c r="C50" t="n">
         <v>44</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>서바이브</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=838594&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>838594</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:27</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="b">
-        <v>1</v>
-      </c>
-      <c r="J49" t="inlineStr">
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:24</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="b">
+        <v>1</v>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N49" t="n">
+      <c r="N50" t="n">
         <v>2</v>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>연금술 무인도 서바이브</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P50" t="inlineStr">
         <is>
           <t>연금술 무인도 서바이브 (총 42화/완결)</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
+      <c r="Q50" t="inlineStr">
         <is>
           <t>총 42화/완결</t>
         </is>
       </c>
-      <c r="R49" t="n">
+      <c r="R50" t="n">
         <v>42</v>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="S50" t="inlineStr">
         <is>
           <t>완결</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>평점 9.9 | 호시 렌지,이구치 콘 호시 렌지 | 2025.02.24. | 총42화/완결 | 1화 무료</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>평점 9.9 | 호시 렌지,이구치 콘 호시 렌지 | 2025.02.24. | 총42화/완결 | 1화 무료</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr">
+      <c r="V50" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=10375934</t>
         </is>
       </c>
-      <c r="W49" t="inlineStr">
+      <c r="W50" t="inlineStr">
         <is>
           <t>10375934</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>연금술 무인도 서바이브 (총 42화/완결)
 평점
@@ -8089,161 +8257,161 @@
 항행 중 사고를 당한 연금술사 니코, 요리사 진, 포로남 셋이 표착한 곳은…… 지도에도 표시돼 있지 않은 무인도였다! 「무인도에서 처음으로 해야 할 일은?」, 「물 확보는 어떻게?」, 「식량 수집의 포인트는?」 살아남기 ..</t>
         </is>
       </c>
-      <c r="Y49" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z49" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA49" t="n">
+      <c r="Y50" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z50" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA50" t="n">
         <v>100</v>
       </c>
-      <c r="AB49" t="inlineStr">
+      <c r="AB50" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_2</t>
         </is>
       </c>
-      <c r="AC49" t="inlineStr">
+      <c r="AC50" t="inlineStr">
         <is>
           <t>matched</t>
         </is>
       </c>
-      <c r="AD49" t="inlineStr">
+      <c r="AD50" t="inlineStr">
         <is>
           <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
-      <c r="AE49" t="n">
+      <c r="AE50" t="n">
         <v>2</v>
       </c>
-      <c r="AF49" t="inlineStr">
+      <c r="AF50" t="inlineStr">
         <is>
           <t>5.6천</t>
         </is>
       </c>
-      <c r="AG49" t="n">
+      <c r="AG50" t="n">
         <v>5600</v>
       </c>
-      <c r="AH49" t="inlineStr">
+      <c r="AH50" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="AI49" t="inlineStr">
+      <c r="AI50" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ49" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK49" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ50" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C50" t="n">
+      <c r="C51" t="n">
         <v>46</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>화스트 페이스</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=847905&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>847905</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:28</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="b">
-        <v>1</v>
-      </c>
-      <c r="J50" t="inlineStr">
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:24</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="b">
+        <v>1</v>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M51" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N50" t="n">
-        <v>1</v>
-      </c>
-      <c r="O50" t="inlineStr">
+      <c r="N51" t="n">
+        <v>1</v>
+      </c>
+      <c r="O51" t="inlineStr">
         <is>
           <t>화스트 페이스</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="P51" t="inlineStr">
         <is>
           <t>화스트 페이스 (총 24화/미완결)</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr">
+      <c r="Q51" t="inlineStr">
         <is>
           <t>총 24화/미완결</t>
         </is>
       </c>
-      <c r="R50" t="n">
+      <c r="R51" t="n">
         <v>24</v>
       </c>
-      <c r="S50" t="inlineStr">
+      <c r="S51" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr">
+      <c r="T51" t="inlineStr">
         <is>
           <t>평점 9.9 | NO_Teamkill NO_Teamkill | 2026.06.13. | 총24화/미완결 | 20화 무료</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="U51" t="inlineStr">
         <is>
           <t>평점 9.9 | NO_Teamkill NO_Teamkill | 2026.06.13. | 총24화/미완결 | 20화 무료</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr">
+      <c r="V51" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=13750354</t>
         </is>
       </c>
-      <c r="W50" t="inlineStr">
+      <c r="W51" t="inlineStr">
         <is>
           <t>13750354</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>화스트 페이스 (총 24화/미완결)
 평점
@@ -8251,155 +8419,155 @@
 화스트 페이스! 상황 발생! 상황 발생!현재 적 대규모 도발로 인해 준전시상태 돌입!전 병력 전투 장비 구비하고 즉각 출동 준비할 수 있도록!제1부 화스트페이스!제2부 20XX년 XX월 XX일 21시44분!제3부 발령권자 군단장!..</t>
         </is>
       </c>
-      <c r="Y50" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z50" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA50" t="n">
+      <c r="Y51" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z51" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA51" t="n">
         <v>105</v>
       </c>
-      <c r="AB50" t="inlineStr">
+      <c r="AB51" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC50" t="inlineStr">
+      <c r="AC51" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD50" t="inlineStr">
+      <c r="AD51" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF50" t="inlineStr"/>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr">
+      <c r="AE51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI50" t="inlineStr">
+      <c r="AI51" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ50" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK50" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ51" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C51" t="n">
+      <c r="C52" t="n">
         <v>79</v>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>사내 계약 연애</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=842148&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>842148</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:29</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="b">
-        <v>1</v>
-      </c>
-      <c r="J51" t="inlineStr">
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:25</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="b">
+        <v>1</v>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr">
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N51" t="n">
-        <v>1</v>
-      </c>
-      <c r="O51" t="inlineStr">
+      <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" t="inlineStr">
         <is>
           <t>사내 계약 연애</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>사내 계약 연애 (총 48화/미완결)</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr">
+      <c r="Q52" t="inlineStr">
         <is>
           <t>총 48화/미완결</t>
         </is>
       </c>
-      <c r="R51" t="n">
+      <c r="R52" t="n">
         <v>48</v>
       </c>
-      <c r="S51" t="inlineStr">
+      <c r="S52" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr">
+      <c r="T52" t="inlineStr">
         <is>
           <t>평점 9.9 | 최무탁, 미리엄 울 | 2026.06.13. | 총48화/미완결 | 42화 무료</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>평점 9.9 | 최무탁, 미리엄 울 | 2026.06.13. | 총48화/미완결 | 42화 무료</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr">
+      <c r="V52" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=13046250</t>
         </is>
       </c>
-      <c r="W51" t="inlineStr">
+      <c r="W52" t="inlineStr">
         <is>
           <t>13046250</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>사내 계약 연애 (총 48화/미완결)
 평점
@@ -8407,161 +8575,161 @@
 예쁘고 잘생긴 것, '미'를 애정하는 서윤.그리고 그런 그녀가 더 애정하는 것은바로 미의 남녀가 서로를 사랑스럽게 탐하는 19금 만화책!그런데 이 미적 추구미에 도달하는 남자가가장 가까이에 그녀의 직속 상사로 있었으니.....</t>
         </is>
       </c>
-      <c r="Y51" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z51" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA51" t="n">
+      <c r="Y52" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z52" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA52" t="n">
         <v>105</v>
       </c>
-      <c r="AB51" t="inlineStr">
+      <c r="AB52" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC51" t="inlineStr">
+      <c r="AC52" t="inlineStr">
         <is>
           <t>matched</t>
         </is>
       </c>
-      <c r="AD51" t="inlineStr">
+      <c r="AD52" t="inlineStr">
         <is>
           <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
-      <c r="AE51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF51" t="inlineStr">
+      <c r="AE52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF52" t="inlineStr">
         <is>
           <t>51.5만</t>
         </is>
       </c>
-      <c r="AG51" t="n">
+      <c r="AG52" t="n">
         <v>515000</v>
       </c>
-      <c r="AH51" t="inlineStr">
+      <c r="AH52" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="AI51" t="inlineStr">
+      <c r="AI52" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ51" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK51" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ52" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C52" t="n">
-        <v>80</v>
-      </c>
-      <c r="D52" t="inlineStr">
+      <c r="C53" t="n">
+        <v>83</v>
+      </c>
+      <c r="D53" t="inlineStr">
         <is>
           <t>나는 참지 못한다</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=823476&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>823476</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:29</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="b">
-        <v>1</v>
-      </c>
-      <c r="J52" t="inlineStr">
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:25</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="b">
+        <v>1</v>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M53" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N52" t="n">
-        <v>1</v>
-      </c>
-      <c r="O52" t="inlineStr">
+      <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" t="inlineStr">
         <is>
           <t>나는 참지 못한다</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="P53" t="inlineStr">
         <is>
           <t>나는 참지 못한다 (총 115화/미완결)</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr">
+      <c r="Q53" t="inlineStr">
         <is>
           <t>총 115화/미완결</t>
         </is>
       </c>
-      <c r="R52" t="n">
+      <c r="R53" t="n">
         <v>115</v>
       </c>
-      <c r="S52" t="inlineStr">
+      <c r="S53" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr">
+      <c r="T53" t="inlineStr">
         <is>
           <t>평점 10.0 | 성현 성현 | 2026.06.13. | 총115화/미완결 | 111화 무료</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="U53" t="inlineStr">
         <is>
           <t>평점 10.0 | 성현 성현 | 2026.06.13. | 총115화/미완결 | 111화 무료</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr">
+      <c r="V53" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=10970308</t>
         </is>
       </c>
-      <c r="W52" t="inlineStr">
+      <c r="W53" t="inlineStr">
         <is>
           <t>10970308</t>
         </is>
       </c>
-      <c r="X52" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>나는 참지 못한다 (총 115화/미완결)
 평점
@@ -8569,155 +8737,155 @@
 평범한 회사원 김연지는 교통사고 이후 변화를 겪게 된다.스트레스가 폭발하면 아무것도 참지 못하는 상태가 되고 만다.계속 일어나는 통제불능 사건들, 자신에게 접근하는 의문의 남성 민성훈.사건은 커지고 일상은 꼬여만 가..</t>
         </is>
       </c>
-      <c r="Y52" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z52" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA52" t="n">
+      <c r="Y53" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z53" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA53" t="n">
         <v>105</v>
       </c>
-      <c r="AB52" t="inlineStr">
+      <c r="AB53" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC52" t="inlineStr">
+      <c r="AC53" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD52" t="inlineStr">
+      <c r="AD53" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF52" t="inlineStr"/>
-      <c r="AG52" t="inlineStr"/>
-      <c r="AH52" t="inlineStr">
+      <c r="AE53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF53" t="inlineStr"/>
+      <c r="AG53" t="inlineStr"/>
+      <c r="AH53" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI52" t="inlineStr">
+      <c r="AI53" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ52" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK52" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ53" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C53" t="n">
-        <v>88</v>
-      </c>
-      <c r="D53" t="inlineStr">
+      <c r="C54" t="n">
+        <v>91</v>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>죽거나 혹은 사랑에 빠지거나</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=819696&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>819696</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>2026-06-22 11:41:29</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="b">
-        <v>1</v>
-      </c>
-      <c r="J53" t="inlineStr">
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:06:26</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="b">
+        <v>1</v>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N53" t="n">
-        <v>1</v>
-      </c>
-      <c r="O53" t="inlineStr">
+      <c r="N54" t="n">
+        <v>1</v>
+      </c>
+      <c r="O54" t="inlineStr">
         <is>
           <t>죽거나 혹은 사랑에 빠지거나</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="P54" t="inlineStr">
         <is>
           <t>죽거나 혹은 사랑에 빠지거나 (총 128화/미완결)</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr">
+      <c r="Q54" t="inlineStr">
         <is>
           <t>총 128화/미완결</t>
         </is>
       </c>
-      <c r="R53" t="n">
+      <c r="R54" t="n">
         <v>128</v>
       </c>
-      <c r="S53" t="inlineStr">
+      <c r="S54" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>평점 9.8 | 허니비 허니비 | 2026.06.13. | 총128화/미완결 | 122화 무료</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t>평점 9.8 | 허니비 허니비 | 2026.06.13. | 총128화/미완결 | 122화 무료</t>
         </is>
       </c>
-      <c r="V53" t="inlineStr">
+      <c r="V54" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=10555314</t>
         </is>
       </c>
-      <c r="W53" t="inlineStr">
+      <c r="W54" t="inlineStr">
         <is>
           <t>10555314</t>
         </is>
       </c>
-      <c r="X53" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>죽거나 혹은 사랑에 빠지거나 (총 128화/미완결)
 평점
@@ -8725,51 +8893,51 @@
 아름다운 도시 루베른에서 일어나는 의문의 연쇄살인 사건. 조용하고 눈에 띄지 않는 이자벨라에게 살인마의 초대장이 전달되는데.. 목숨을 건 15일간의 내기. 절대 어떤 쾌락과 환상에도 사랑에 빠져서는 안 된다.</t>
         </is>
       </c>
-      <c r="Y53" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z53" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA53" t="n">
+      <c r="Y54" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z54" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA54" t="n">
         <v>105</v>
       </c>
-      <c r="AB53" t="inlineStr">
+      <c r="AB54" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC53" t="inlineStr">
+      <c r="AC54" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD53" t="inlineStr">
+      <c r="AD54" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE53" t="n">
+      <c r="AE54" t="n">
         <v>2</v>
       </c>
-      <c r="AF53" t="inlineStr"/>
-      <c r="AG53" t="inlineStr"/>
-      <c r="AH53" t="inlineStr">
+      <c r="AF54" t="inlineStr"/>
+      <c r="AG54" t="inlineStr"/>
+      <c r="AH54" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI53" t="inlineStr">
+      <c r="AI54" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ53" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK53" t="inlineStr">
-        <is>
-          <t>2026-06-22 12:22:39</t>
+      <c r="AJ54" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:48:27</t>
         </is>
       </c>
     </row>

</xml_diff>